<commit_message>
S2 Week 2: write Logs with FileLog/ErrorAlert flags, email runtime failures with who/when/where/browser/device, grant Tufan_Doctor extra menus without other-clinic case access, and use tufanpowar001@gmail.com on Dev seeds.
</commit_message>
<xml_diff>
--- a/ScriptsAndFiles/Homeocentrum_All_New_And_Updated+APIs.xlsx
+++ b/ScriptsAndFiles/Homeocentrum_All_New_And_Updated+APIs.xlsx
@@ -12894,12 +12894,12 @@
       <c r="O115" s="6" t="inlineStr"/>
       <c r="P115" s="6" t="inlineStr">
         <is>
-          <t>Clinic login. Reception token now includes RoleName=Reception and DoctorUserID (owning doctor's UserMaster id) for New-API backup/ACL.</t>
+          <t>Clinic login. Reception token includes RoleName=Reception, DoctorID, and doctorUserId (owning doctor's UserMaster id) for New-API dashboard stats. PatientBoardBackup stays DoctorOnly 403.</t>
         </is>
       </c>
       <c r="Q115" s="6" t="inlineStr">
         <is>
-          <t>{ "userName": "tufanpowar001@gmail.com", "password": "123456" }</t>
+          <t>{ "userName": "Tufan_Reception", "password": "123456" }</t>
         </is>
       </c>
       <c r="R115" s="6" t="inlineStr">
@@ -26422,12 +26422,12 @@
       <c r="O51" s="6" t="inlineStr"/>
       <c r="P51" s="6" t="inlineStr">
         <is>
-          <t>Clinic login. Reception token now includes RoleName=Reception and DoctorUserID (owning doctor's UserMaster id) for New-API backup/ACL.</t>
+          <t>Clinic login. Reception token includes RoleName=Reception, DoctorID, and doctorUserId (owning doctor's UserMaster id) for New-API dashboard stats. PatientBoardBackup stays DoctorOnly 403.</t>
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>{ "userName": "tufanpowar001@gmail.com", "password": "123456" }</t>
+          <t>{ "userName": "Tufan_Reception", "password": "123456" }</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -51923,12 +51923,12 @@
       <c r="O50" s="6" t="inlineStr"/>
       <c r="P50" s="6" t="inlineStr">
         <is>
-          <t>Clinic login. Reception token now includes RoleName=Reception and DoctorUserID (owning doctor's UserMaster id) for New-API backup/ACL.</t>
+          <t>Clinic login. Reception token includes RoleName=Reception, DoctorID, and doctorUserId (owning doctor's UserMaster id) for New-API dashboard stats. PatientBoardBackup stays DoctorOnly 403.</t>
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>{ "userName": "tufanpowar001@gmail.com", "password": "123456" }</t>
+          <t>{ "userName": "Tufan_Reception", "password": "123456" }</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">

</xml_diff>